<commit_message>
Reorganiza perfis em 2 setores e adiciona unidade de medida ao produto
- Tela de perfil com dois setores: Vendas (azul) e Gestão (verde). Jeovana e
  Reginaldo deixam de ser gerência-leitura e passam a Gestão geral (veem as
  duas lojas, consultam e respondem). "Gestão geral (você)" vira "Ciça".
- Produtos ganham unidade de medida (coluna `unidade` na aba Produtos e no
  mock). Ao escolher o produto, a unidade já vem pré-selecionada no pedido do
  vendedor e aparece na descrição (também na Consulta da Gestão). Novas opções
  de unidade: sc e lata.
- Codigo.gs lê a coluna C (unidade); planilha pronta, README e PLANILHA.md
  atualizados. Compatível com planilhas sem a coluna (unidade fica em branco).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DShXxKe35WYbd9tYbq28CA
</commit_message>
<xml_diff>
--- a/estoque-chrome/apps-script/planilha/Estoque-Portal-Timoni.xlsx
+++ b/estoque-chrome/apps-script/planilha/Estoque-Portal-Timoni.xlsx
@@ -427,11 +427,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,6 +446,11 @@
           <t>descricao</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>unidade</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -457,6 +463,11 @@
           <t>Torneira monocomando cozinha cromada</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -469,6 +480,11 @@
           <t>Torneira parede jardim 1/2 polegada</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -481,6 +497,11 @@
           <t>Registro de gaveta 3/4 bruto</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -493,6 +514,11 @@
           <t>Registro de pressão 1/2 cromado</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -505,6 +531,11 @@
           <t>Tubo PVC soldável 25mm 6m</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -517,6 +548,11 @@
           <t>Tubo PVC esgoto 100mm 6m</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>barra</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -529,6 +565,11 @@
           <t>Joelho 90 graus PVC soldável 25mm</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -541,6 +582,11 @@
           <t>Cimento CP II 50kg</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>sc</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -553,6 +599,11 @@
           <t>Argamassa colante AC II 20kg</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>sc</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -565,6 +616,11 @@
           <t>Disjuntor bipolar 32A</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -577,6 +633,11 @@
           <t>Disjuntor monopolar 20A</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -589,6 +650,11 @@
           <t>Cabo flexível 2,5mm preto 100m</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rolo</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -601,6 +667,11 @@
           <t>Tinta acrílica branca 18L</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>lata</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -613,6 +684,11 @@
           <t>Tinta esmalte sintético branco 3,6L</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>lata</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -623,6 +699,11 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>Vaso sanitário com caixa acoplada branco</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>un</t>
         </is>
       </c>
     </row>

</xml_diff>